<commit_message>
Add product list keyed to campaign sequence
Adds a Products sheet and CSV listing the hero, bundle add-on, cross-sell
and upsell SKU for each campaign in order, with variant, SKU, live price,
stock, storefront URL and the reason for the pick.

Flags a name collision: three products share the Kalash Khazana name and
only the 1249 two-and-a-half-inch one is the campaign SKU.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjSU6dDwFBwk34LrSdddTP
</commit_message>
<xml_diff>
--- a/campaigns/Dev-Aastha-WhatsApp-Campaigns.xlsx
+++ b/campaigns/Dev-Aastha-WhatsApp-Campaigns.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaigns" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offers &amp; Send Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offers &amp; Send Plan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Campaigns'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Products'!$A$1:$J$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +90,23 @@
       <color rgb="FF1C1917"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="8"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF78716C"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -138,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -200,6 +219,36 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1296,6 +1345,959 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="9" max="9"/>
+    <col width="54" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Variant</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Price (₹)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Product URL</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Why this product</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="46" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>PDP Visit 15–30 Days</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="inlineStr">
+        <is>
+          <t>Dev Aastha Silver Plated Kuber Kalash Khazana | Laxmi Murti</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>2.5 inch</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Dev-SP- Kalash Khazana -2.55 inch</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="n">
+        <v>1249</v>
+      </c>
+      <c r="H2" s="24" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="I2" s="25" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/silver-plated-kalash-khazana-2-5-inch</t>
+        </is>
+      </c>
+      <c r="J2" s="26" t="inlineStr">
+        <is>
+          <t>#1 by order count — 203 orders in 30 days. Lowest price barrier in the catalogue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="22" t="inlineStr"/>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>BUNDLE ADD-ON</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="inlineStr">
+        <is>
+          <t>Lakshmi Charan Silver-Plated Idol</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>3 inch</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>DEV-SP-Lakshmi Charan W(Base) - 3 Inch</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="n">
+        <v>1499</v>
+      </c>
+      <c r="H3" s="24" t="inlineStr">
+        <is>
+          <t>453</t>
+        </is>
+      </c>
+      <c r="I3" s="25" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/lakshmi-charan-silver-plated-idol</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="inlineStr">
+        <is>
+          <t>Takes cart to ₹2,748, clearing the ₹1,999 floor for LAKSHMI251.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>PDP Visit 7–14 Days</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>DYNAMIC — the exact product they viewed</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>as viewed</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="inlineStr"/>
+      <c r="J4" s="31" t="inlineStr">
+        <is>
+          <t>Recent intent. Re-show what they looked at, do not switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="27" t="inlineStr"/>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>CROSS-SELL</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Dev Aastha Silver Plated Kuber Kalash Khazana | Laxmi Murti</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>2.5 inch</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Dev-SP- Kalash Khazana -2.55 inch</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>1249</v>
+      </c>
+      <c r="H5" s="29" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="I5" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/silver-plated-kalash-khazana-2-5-inch</t>
+        </is>
+      </c>
+      <c r="J5" s="31" t="inlineStr">
+        <is>
+          <t>Carries the 200+ orders proof point that the copy leans on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>PDP Visit 2–7 Days</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>DYNAMIC — the exact product they viewed</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>as viewed</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="25" t="inlineStr"/>
+      <c r="J6" s="26" t="inlineStr">
+        <is>
+          <t>Hottest cohort. Pure re-show, no cross-sell, no discount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Coll Visit – 180 Days</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Silver-Plated Lakshmi Ganesha Idol Set | Auspicious Ganesh Laxmi Murti</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>3.7 inch</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>DEV-SP- Lakshmi Ganesh - 3.7 Inch</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>2499</v>
+      </c>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/lakshmi-ganesh-silver-plated-idol-set</t>
+        </is>
+      </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>59 sets in 30 days at ₹2,743 AOV. Existing velvet-box asset ready to use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="27" t="inlineStr"/>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>BUNDLE ADD-ON</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Panchmukhi Diya Silver-Plated for Pooja</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>DEV-PANCHMUKHI_DIYA</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>1999</v>
+      </c>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+      <c r="I8" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/panchmukhi-diya-silver-plated-for-pooja</t>
+        </is>
+      </c>
+      <c r="J8" s="31" t="inlineStr">
+        <is>
+          <t>Takes cart to ₹4,498, clearing the ₹2,999 floor for SET351.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>HP Visit 7–30 Days</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Handcrafted Silver-Plated Elephant Pair for Vastu &amp; Gifting</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>2 Inch</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DEV-SP-P(2)-ELEPENT-2INCH</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>1499</v>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>322</t>
+        </is>
+      </c>
+      <c r="I9" s="25" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/elephant-murti-silver-plated</t>
+        </is>
+      </c>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t>#1 by revenue — 533 orders in 180 days. Entry price equals the ₹1,499 floor exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="22" t="inlineStr"/>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>UPSELL LADDER</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Elephant Pair — larger sizes</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>3in ₹2,099 · 4in ₹3,499 · 5in ₹6,999 · 7in ₹10,999</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>DEV-SP-P(2)-ELEPENT-3/4/5/7INCH</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>2099-10999</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>442/489/499/498</t>
+        </is>
+      </c>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/elephant-murti-silver-plated</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="inlineStr">
+        <is>
+          <t>Show on the PDP, not in the message. Keeps the ₹1,499 hook clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>Orders – 180 Days</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>Lakshmi Charan Silver-Plated Idol</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>3 inch</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>DEV-SP-Lakshmi Charan W(Base) - 3 Inch</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>1499</v>
+      </c>
+      <c r="H11" s="29" t="inlineStr">
+        <is>
+          <t>453</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/lakshmi-charan-silver-plated-idol</t>
+        </is>
+      </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>Completion logic: they already own Ganesha. No discount — early access only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="27" t="inlineStr"/>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>UPSELL</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Lakshmi Charan Silver-Plated Idol</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>5 inch</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>DEV-SP-Lakshmi Charan W(Base) - 5 Inch</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>2499</v>
+      </c>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>496</t>
+        </is>
+      </c>
+      <c r="I12" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/lakshmi-charan-silver-plated-idol</t>
+        </is>
+      </c>
+      <c r="J12" s="31" t="inlineStr">
+        <is>
+          <t>Repeat buyers trade up. Averaged ₹9,857/order last month — bulk demand is real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>ATC – 180 Days</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>DYNAMIC — the exact product in their cart</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>as in cart</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="25" t="inlineStr"/>
+      <c r="J13" s="26" t="inlineStr">
+        <is>
+          <t>Never substitute a cart item. Show back exactly what they chose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>Orders 180d — bulk slice</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>HERO</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Silver Plated Shubh Labh Door Decor for Home Entrance - 5 Inch</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Pack of 6</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>DEV-SP- BandarWal– 4.5-inch P(6)</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>7499</v>
+      </c>
+      <c r="H14" s="29" t="inlineStr">
+        <is>
+          <t>498</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/silver-plated-subh-labh-hanging-4-5-inch</t>
+        </is>
+      </c>
+      <c r="J14" s="31" t="inlineStr">
+        <is>
+          <t>₹1,250 per piece. Clears the ₹7,499 floor for BULK1100 on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="27" t="inlineStr"/>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>ALSO OFFER</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Shubh Labh — Single · Kuber Kalash · Lakshmi Charan 3in</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Single ₹2,999 · ₹1,249 · ₹1,499</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>DEV-SP- Shubh Labh - 4.5 Inch + 2 others</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>1249-2999</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="inlineStr">
+        <is>
+          <t>486/531/453</t>
+        </is>
+      </c>
+      <c r="I15" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/silver-plated-subh-labh-hanging-4-5-inch</t>
+        </is>
+      </c>
+      <c r="J15" s="31" t="inlineStr">
+        <is>
+          <t>Mix-and-match options for buyers building a list to a headcount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>ALL — Pitru Paksha</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>NO PRODUCT</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>No product in the message — pre-book only</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="25" t="inlineStr"/>
+      <c r="J16" s="26" t="inlineStr">
+        <is>
+          <t>Selling murtis during Shraddh is the one thing that damages trust here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="22" t="inlineStr"/>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>RESERVE LIST (goes live 11 Oct)</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>Kuber Kalash · Ashta Lakshmi Tortoise 2in · Panchmukhi Diya</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>₹1,249 · ₹1,499 · ₹1,999</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Kalash 2.55 + Ashta 2in + PANCHMUKHI_DIYA</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr">
+        <is>
+          <t>1249-1999</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>531/488/514</t>
+        </is>
+      </c>
+      <c r="I17" s="25" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/ashta-lakshmi-tortoise-silver-plated-idol</t>
+        </is>
+      </c>
+      <c r="J17" s="26" t="inlineStr">
+        <is>
+          <t>Ghatasthapana set. Reserve now, charge on 11 Oct when Navratri opens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>ALL — Dhanteras</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>HERO (combo)</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Lakshmi Charan 3in + Kuber Kalash 2.5in</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>₹1,499 + ₹1,249 = ₹2,748</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Lakshmi Charan 3 Inch + Kalash Khazana 2.55 inch</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>2748</v>
+      </c>
+      <c r="H18" s="29" t="inlineStr">
+        <is>
+          <t>453/531</t>
+        </is>
+      </c>
+      <c r="I18" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/lakshmi-charan-silver-plated-idol</t>
+        </is>
+      </c>
+      <c r="J18" s="31" t="inlineStr">
+        <is>
+          <t>Both wealth heroes in one cart. ₹251 off lands it at ₹2,497.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="27" t="inlineStr"/>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>ALSO PUSH</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Ashta Lakshmi Tortoise · Lakshmi Ganesha Set</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>2in ₹1,499 / 4.5in ₹3,299 · Set ₹2,499</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Ashta Lakshmi 2in/4.5in + Lakshmi Ganesh 3.7</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>1499-3299</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="inlineStr">
+        <is>
+          <t>488/491/403</t>
+        </is>
+      </c>
+      <c r="I19" s="30" t="inlineStr">
+        <is>
+          <t>https://www.devaastha.com/products/ashta-lakshmi-tortoise-silver-plated-idol</t>
+        </is>
+      </c>
+      <c r="J19" s="31" t="inlineStr">
+        <is>
+          <t>Dhanteras is a buy-silver day, not a one-SKU day. Give the mandir a full shelf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>NOTES ON PRODUCT SELECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>NAME COLLISION — there are three "Kalash Khazana" products. The campaign SKU is the ₹1,249 one: "Dev Aastha Silver Plated Kuber Kalash Khazana | Laxmi Murti", handle silver-plated-kalash-khazana-2-5-inch, SKU "Dev-SP- Kalash Khazana -2.55 inch". Do NOT use the 4.5-inch ₹3,499 version or the draft ₹3,499 one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>EXCLUDE FROM ALL SENDS — Standing Hanuman 5.5" is at 0 stock; Balaji 6" and 8" variants are at 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Ganesh SKUs are deliberately absent. Visarjan was 25 Sep, so Divine Ganesha, Throne Ganesha and Trishul Ganesh have no occasion behind them until next year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Every bundle add-on exists to clear a cart minimum. Remove the add-on and the flat discount becomes a straight margin loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Prices and stock pulled live from Shopify on 24 September 2026. Re-check stock the morning of each send.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J19"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId14"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>